<commit_message>
Entrenar y documentar seis modelos reales
</commit_message>
<xml_diff>
--- a/reports/reporte_resultados_modelos.xlsx
+++ b/reports/reporte_resultados_modelos.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2e3a6cf5b7264e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDA_Clases" sheetId="2" r:id="R7a0f198a21954c73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDA_Estadisticos" sheetId="3" r:id="R74b286d6d53e46d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparacion_Modelos" sheetId="4" r:id="R899fd3c453d748c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CV_5_Folds" sheetId="5" r:id="R6509224817c54f4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CV_Resumen" sheetId="6" r:id="R8b03264808da40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning" sheetId="7" r:id="R50a965996102411e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friedman" sheetId="8" r:id="R473c371c9065428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wilcoxon_Holm" sheetId="9" r:id="Rb8b6eb94df64467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MLP_TFIDF" sheetId="10" r:id="R9f3aac8d39414c61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CNN_1D" sheetId="11" r:id="R2f9b99228c7a43e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LSTM" sheetId="12" r:id="Rb935a37f5162456c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CNN_BiLSTM" sheetId="13" r:id="R1435772a77f24f33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BiLSTM_Atencion" sheetId="14" r:id="R475708eb8e6f451f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="15" r:id="R2dafc8c1318a44cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R21ae7a3403e04397"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDA_Clases" sheetId="2" r:id="Rf2389986423e4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EDA_Estadisticos" sheetId="3" r:id="R00c16727d30a4b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparacion_Modelos" sheetId="4" r:id="Rf39c6cbd2353492c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CV_5_Folds" sheetId="5" r:id="Rbc4fe62cc2e544d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CV_Resumen" sheetId="6" r:id="R8f31222a507847ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuning" sheetId="7" r:id="R79e678b74c304771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friedman" sheetId="8" r:id="R42728a3304464dc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wilcoxon_Holm" sheetId="9" r:id="R8a28ca1fa71b46a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MLP_TFIDF" sheetId="10" r:id="R009b8d6221a7405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CNN_1D" sheetId="11" r:id="R15df651b308d48ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LSTM" sheetId="12" r:id="Ra45bc8817d2444e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CNN_BiLSTM" sheetId="13" r:id="R1578409b1b354142"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BiLSTM_Atencion" sheetId="14" r:id="R146b479f44484805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="15" r:id="Rb673b2050e504aaf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BiLSTM" sheetId="16" r:id="Rc564258eb94a4676"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -66,7 +67,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -88,15 +89,43 @@
         <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF16324F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F75B5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="5">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -217,6 +246,50 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -236,17 +309,14 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr/>
               <a:t>Métricas por modelo</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:varyColors val="0"/>
@@ -258,7 +328,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Comparacion_Modelos'!$A$4:$A$8</c:f>
+              <c:f>'Comparacion_Modelos'!$A$4:$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -266,7 +336,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comparacion_Modelos'!$B$4:$B$8</c:f>
+              <c:f>'Comparacion_Modelos'!$B$4:$B$9</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -282,7 +352,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Comparacion_Modelos'!$A$4:$A$8</c:f>
+              <c:f>'Comparacion_Modelos'!$A$4:$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -290,7 +360,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comparacion_Modelos'!$C$4:$C$8</c:f>
+              <c:f>'Comparacion_Modelos'!$C$4:$C$9</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -306,7 +376,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Comparacion_Modelos'!$A$4:$A$8</c:f>
+              <c:f>'Comparacion_Modelos'!$A$4:$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -314,7 +384,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comparacion_Modelos'!$D$4:$D$8</c:f>
+              <c:f>'Comparacion_Modelos'!$D$4:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -330,7 +400,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Comparacion_Modelos'!$A$4:$A$8</c:f>
+              <c:f>'Comparacion_Modelos'!$A$4:$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -338,7 +408,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Comparacion_Modelos'!$E$4:$E$8</c:f>
+              <c:f>'Comparacion_Modelos'!$E$4:$E$9</c:f>
               <c:numCache>
                 <c:formatCode>0.0000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -453,7 +523,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1416dab4e1f04fbd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R079ae48b22ce47eb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -511,7 +581,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TablaComparacionModelos" displayName="TablaComparacionModelos" ref="A3:M8" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TablaComparacionModelos" displayName="TablaComparacionModelos" ref="A3:M9" headerRowCount="1" totalsRowCount="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="modelo"/>
     <x:tableColumn id="2" name="accuracy"/>
@@ -654,9 +724,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -843,7 +913,7 @@
         <x:v>Modelos comparados</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>ROC AUC macro</x:v>
@@ -868,7 +938,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="27" t="str">
-        <x:v>Interpretación: MLP-TFIDF alcanzó el mayor F1 macro en el conjunto oficial de prueba. La prueba de Friedman detectó diferencias globales entre los cinco modelos (p &lt; 0,05); las comparaciones pareadas Wilcoxon-Holm no fueron significativas con solo cinco folds.</x:v>
+        <x:v>Interpretación: MLP-TFIDF alcanzó el mayor F1 macro en el conjunto oficial de prueba. La comparación test incluye seis modelos: tres base y tres híbridos. La prueba de Friedman se conserva sobre los cinco modelos evaluados por validación cruzada (p &lt; 0,05); las comparaciones pareadas Wilcoxon-Holm no fueron significativas con cinco folds.</x:v>
       </x:c>
       <x:c r="B10" s="27"/>
       <x:c r="C10" s="27"/>
@@ -2192,6 +2262,194 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25" customHeight="1">
+      <x:c r="A1" s="54" t="str">
+        <x:v>Reporte por clase - BiLSTM</x:v>
+      </x:c>
+      <x:c r="B1" s="54"/>
+      <x:c r="C1" s="54"/>
+      <x:c r="D1" s="54"/>
+      <x:c r="E1" s="54"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="59" t="str">
+        <x:v>clase</x:v>
+      </x:c>
+      <x:c r="B3" s="59" t="str">
+        <x:v>precision</x:v>
+      </x:c>
+      <x:c r="C3" s="59" t="str">
+        <x:v>recall</x:v>
+      </x:c>
+      <x:c r="D3" s="59" t="str">
+        <x:v>f1-score</x:v>
+      </x:c>
+      <x:c r="E3" s="59" t="str">
+        <x:v>support</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="64" t="str">
+        <x:v>Declaración</x:v>
+      </x:c>
+      <x:c r="B4" s="67" t="str">
+        <x:v>0.8338928856914468</x:v>
+      </x:c>
+      <x:c r="C4" s="67" t="str">
+        <x:v>0.5884476534296029</x:v>
+      </x:c>
+      <x:c r="D4" s="67" t="str">
+        <x:v>0.6899927243865335</x:v>
+      </x:c>
+      <x:c r="E4" s="67" t="str">
+        <x:v>8864.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="65" t="str">
+        <x:v>Pregunta declarativa</x:v>
+      </x:c>
+      <x:c r="B5" s="68" t="str">
+        <x:v>0.38556618819776717</x:v>
+      </x:c>
+      <x:c r="C5" s="68" t="str">
+        <x:v>0.43054318788958146</x:v>
+      </x:c>
+      <x:c r="D5" s="68" t="str">
+        <x:v>0.40681531342027766</x:v>
+      </x:c>
+      <x:c r="E5" s="68" t="str">
+        <x:v>2246.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="65" t="str">
+        <x:v>Retroalimentación breve</x:v>
+      </x:c>
+      <x:c r="B6" s="68" t="str">
+        <x:v>0.6118175018698578</x:v>
+      </x:c>
+      <x:c r="C6" s="68" t="str">
+        <x:v>0.8342682304946456</x:v>
+      </x:c>
+      <x:c r="D6" s="68" t="str">
+        <x:v>0.705933117583603</x:v>
+      </x:c>
+      <x:c r="E6" s="68" t="str">
+        <x:v>1961.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="65" t="str">
+        <x:v>Continuación / seguimiento</x:v>
+      </x:c>
+      <x:c r="B7" s="68" t="str">
+        <x:v>0.7313961729270021</x:v>
+      </x:c>
+      <x:c r="C7" s="68" t="str">
+        <x:v>0.7835990888382688</x:v>
+      </x:c>
+      <x:c r="D7" s="68" t="str">
+        <x:v>0.7565982404692082</x:v>
+      </x:c>
+      <x:c r="E7" s="68" t="str">
+        <x:v>1317.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="65" t="str">
+        <x:v>Pregunta</x:v>
+      </x:c>
+      <x:c r="B8" s="68" t="str">
+        <x:v>0.2730739893211289</x:v>
+      </x:c>
+      <x:c r="C8" s="68" t="str">
+        <x:v>0.6617375231053605</x:v>
+      </x:c>
+      <x:c r="D8" s="68" t="str">
+        <x:v>0.38660907127429806</x:v>
+      </x:c>
+      <x:c r="E8" s="68" t="str">
+        <x:v>1082.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="65" t="str">
+        <x:v>accuracy</x:v>
+      </x:c>
+      <x:c r="B9" s="68" t="str">
+        <x:v>0.6184227537168714</x:v>
+      </x:c>
+      <x:c r="C9" s="68" t="str">
+        <x:v>0.6184227537168714</x:v>
+      </x:c>
+      <x:c r="D9" s="68" t="str">
+        <x:v>0.6184227537168714</x:v>
+      </x:c>
+      <x:c r="E9" s="68" t="str">
+        <x:v>0.6184227537168714</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="65" t="str">
+        <x:v>macro avg</x:v>
+      </x:c>
+      <x:c r="B10" s="68" t="str">
+        <x:v>0.5671493476014406</x:v>
+      </x:c>
+      <x:c r="C10" s="68" t="str">
+        <x:v>0.6597191367514919</x:v>
+      </x:c>
+      <x:c r="D10" s="68" t="str">
+        <x:v>0.5891896934267841</x:v>
+      </x:c>
+      <x:c r="E10" s="68" t="str">
+        <x:v>15470.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="66" t="str">
+        <x:v>weighted avg</x:v>
+      </x:c>
+      <x:c r="B11" s="69" t="str">
+        <x:v>0.6927018186695723</x:v>
+      </x:c>
+      <x:c r="C11" s="69" t="str">
+        <x:v>0.6184227537168714</x:v>
+      </x:c>
+      <x:c r="D11" s="69" t="str">
+        <x:v>0.635351547789422</x:v>
+      </x:c>
+      <x:c r="E11" s="69" t="str">
+        <x:v>15470.0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -2300,7 +2558,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R395d1b78a4fa48ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ab59dbc27b24311"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2426,7 +2684,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb16ee9d6fc9d4f9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc64e22f3fa404dc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2452,7 +2710,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="33" t="str">
-        <x:v>Comparación de los cinco modelos</x:v>
+        <x:v>Comparación de los seis modelos</x:v>
       </x:c>
       <x:c r="B1" s="33"/>
       <x:c r="C1" s="33"/>
@@ -2512,40 +2770,40 @@
       <x:c r="A4" s="42" t="str">
         <x:v>MLP-TFIDF</x:v>
       </x:c>
-      <x:c r="B4" s="44" t="n">
+      <x:c r="B4" s="44" t="str">
         <x:v>0.6426632191338074</x:v>
       </x:c>
-      <x:c r="C4" s="44" t="n">
+      <x:c r="C4" s="44" t="str">
         <x:v>0.5983336202056329</x:v>
       </x:c>
-      <x:c r="D4" s="44" t="n">
+      <x:c r="D4" s="44" t="str">
         <x:v>0.6879109753619229</x:v>
       </x:c>
-      <x:c r="E4" s="44" t="n">
+      <x:c r="E4" s="44" t="str">
         <x:v>0.6219238248176198</x:v>
       </x:c>
-      <x:c r="F4" s="44" t="n">
+      <x:c r="F4" s="44" t="str">
         <x:v>0.656718531380011</x:v>
       </x:c>
-      <x:c r="G4" s="44" t="n">
-        <x:v>0.8895966782707448</x:v>
-      </x:c>
-      <x:c r="H4" s="44" t="n">
-        <x:v>1.5864507719998073</x:v>
-      </x:c>
-      <x:c r="I4" s="44" t="n">
-        <x:v>0.0707021459998031</x:v>
-      </x:c>
-      <x:c r="J4" s="44" t="n">
-        <x:v>0.004570274466697</x:v>
-      </x:c>
-      <x:c r="K4" s="44" t="n">
+      <x:c r="G4" s="44" t="str">
+        <x:v>0.8895966715369884</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="str">
+        <x:v>1.556016422000539</x:v>
+      </x:c>
+      <x:c r="I4" s="44" t="str">
+        <x:v>0.056870423002692405</x:v>
+      </x:c>
+      <x:c r="J4" s="44" t="str">
+        <x:v>0.0036761747254487657</x:v>
+      </x:c>
+      <x:c r="K4" s="44" t="str">
         <x:v>1.2569</x:v>
       </x:c>
-      <x:c r="L4" s="44" t="n">
+      <x:c r="L4" s="50" t="str">
         <x:v>328709</x:v>
       </x:c>
-      <x:c r="M4" s="44" t="n">
+      <x:c r="M4" s="50" t="str">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -2553,179 +2811,206 @@
       <x:c r="A5" s="42" t="str">
         <x:v>CNN-1D</x:v>
       </x:c>
-      <x:c r="B5" s="44" t="n">
+      <x:c r="B5" s="44" t="str">
         <x:v>0.6488041370394312</x:v>
       </x:c>
-      <x:c r="C5" s="44" t="n">
-        <x:v>0.5898712855760979</x:v>
-      </x:c>
-      <x:c r="D5" s="44" t="n">
-        <x:v>0.6613919396539257</x:v>
-      </x:c>
-      <x:c r="E5" s="44" t="n">
-        <x:v>0.5977109609590849</x:v>
-      </x:c>
-      <x:c r="F5" s="44" t="n">
-        <x:v>0.65965265704237</x:v>
-      </x:c>
-      <x:c r="G5" s="44" t="n">
-        <x:v>0.8737442136958599</x:v>
-      </x:c>
-      <x:c r="H5" s="44" t="n">
-        <x:v>2.698964734999663</x:v>
-      </x:c>
-      <x:c r="I5" s="44" t="n">
-        <x:v>0.1005147119999492</x:v>
-      </x:c>
-      <x:c r="J5" s="44" t="n">
-        <x:v>0.0064973957336748</x:v>
-      </x:c>
-      <x:c r="K5" s="44" t="n">
+      <x:c r="C5" s="44" t="str">
+        <x:v>0.5899517344164433</x:v>
+      </x:c>
+      <x:c r="D5" s="44" t="str">
+        <x:v>0.6619452627920049</x:v>
+      </x:c>
+      <x:c r="E5" s="44" t="str">
+        <x:v>0.5979479776900531</x:v>
+      </x:c>
+      <x:c r="F5" s="44" t="str">
+        <x:v>0.6596753516651233</x:v>
+      </x:c>
+      <x:c r="G5" s="44" t="str">
+        <x:v>0.8738172479393664</x:v>
+      </x:c>
+      <x:c r="H5" s="44" t="str">
+        <x:v>3.1101645410017227</x:v>
+      </x:c>
+      <x:c r="I5" s="44" t="str">
+        <x:v>0.14751100299326936</x:v>
+      </x:c>
+      <x:c r="J5" s="44" t="str">
+        <x:v>0.009535294311135705</x:v>
+      </x:c>
+      <x:c r="K5" s="44" t="str">
         <x:v>1.376</x:v>
       </x:c>
-      <x:c r="L5" s="44" t="n">
+      <x:c r="L5" s="50" t="str">
         <x:v>359941</x:v>
       </x:c>
-      <x:c r="M5" s="44" t="n">
+      <x:c r="M5" s="50" t="str">
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="42" t="str">
-        <x:v>BiLSTM-Atencion</x:v>
-      </x:c>
-      <x:c r="B6" s="44" t="n">
-        <x:v>0.582223658694247</x:v>
-      </x:c>
-      <x:c r="C6" s="44" t="n">
-        <x:v>0.577555885822121</x:v>
-      </x:c>
-      <x:c r="D6" s="44" t="n">
-        <x:v>0.6703302717545263</x:v>
-      </x:c>
-      <x:c r="E6" s="44" t="n">
-        <x:v>0.5801219649502566</x:v>
-      </x:c>
-      <x:c r="F6" s="44" t="n">
-        <x:v>0.6057413830721956</x:v>
-      </x:c>
-      <x:c r="G6" s="44" t="n">
-        <x:v>0.8768979084474336</x:v>
-      </x:c>
-      <x:c r="H6" s="44" t="n">
-        <x:v>19.697710760000064</x:v>
-      </x:c>
-      <x:c r="I6" s="44" t="n">
-        <x:v>0.6746319379999477</x:v>
-      </x:c>
-      <x:c r="J6" s="44" t="n">
-        <x:v>0.0436090457659953</x:v>
-      </x:c>
-      <x:c r="K6" s="44" t="n">
-        <x:v>1.4949</x:v>
-      </x:c>
-      <x:c r="L6" s="44" t="n">
-        <x:v>390438</x:v>
-      </x:c>
-      <x:c r="M6" s="44" t="n">
+        <x:v>BiLSTM</x:v>
+      </x:c>
+      <x:c r="B6" s="44" t="str">
+        <x:v>0.6184227537168714</x:v>
+      </x:c>
+      <x:c r="C6" s="44" t="str">
+        <x:v>0.5671493476014406</x:v>
+      </x:c>
+      <x:c r="D6" s="44" t="str">
+        <x:v>0.6597191367514919</x:v>
+      </x:c>
+      <x:c r="E6" s="44" t="str">
+        <x:v>0.5891896934267841</x:v>
+      </x:c>
+      <x:c r="F6" s="44" t="str">
+        <x:v>0.635351547789422</x:v>
+      </x:c>
+      <x:c r="G6" s="44" t="str">
+        <x:v>0.8633372628340548</x:v>
+      </x:c>
+      <x:c r="H6" s="44" t="str">
+        <x:v>8.273143267993873</x:v>
+      </x:c>
+      <x:c r="I6" s="44" t="str">
+        <x:v>0.5592023680001148</x:v>
+      </x:c>
+      <x:c r="J6" s="44" t="str">
+        <x:v>0.03614753510020134</x:v>
+      </x:c>
+      <x:c r="K6" s="44" t="str">
+        <x:v>1.4695</x:v>
+      </x:c>
+      <x:c r="L6" s="50" t="str">
+        <x:v>384293</x:v>
+      </x:c>
+      <x:c r="M6" s="50" t="str">
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="42" t="str">
-        <x:v>CNN-BiLSTM</x:v>
-      </x:c>
-      <x:c r="B7" s="44" t="n">
-        <x:v>0.5537168713639302</x:v>
-      </x:c>
-      <x:c r="C7" s="44" t="n">
-        <x:v>0.5539803060668567</x:v>
-      </x:c>
-      <x:c r="D7" s="44" t="n">
-        <x:v>0.6679316258447784</x:v>
-      </x:c>
-      <x:c r="E7" s="44" t="n">
-        <x:v>0.5625670453076338</x:v>
-      </x:c>
-      <x:c r="F7" s="44" t="n">
-        <x:v>0.570664316396819</x:v>
-      </x:c>
-      <x:c r="G7" s="44" t="n">
-        <x:v>0.873439869175705</x:v>
-      </x:c>
-      <x:c r="H7" s="44" t="n">
-        <x:v>15.307453821999843</x:v>
-      </x:c>
-      <x:c r="I7" s="44" t="n">
-        <x:v>0.7327943929999492</x:v>
-      </x:c>
-      <x:c r="J7" s="44" t="n">
-        <x:v>0.0473687390433063</x:v>
-      </x:c>
-      <x:c r="K7" s="44" t="n">
-        <x:v>1.4834</x:v>
-      </x:c>
-      <x:c r="L7" s="44" t="n">
-        <x:v>387445</x:v>
-      </x:c>
-      <x:c r="M7" s="44" t="n">
+        <x:v>BiLSTM-Atencion</x:v>
+      </x:c>
+      <x:c r="B7" s="44" t="str">
+        <x:v>0.5865546218487395</x:v>
+      </x:c>
+      <x:c r="C7" s="44" t="str">
+        <x:v>0.5797487313766385</x:v>
+      </x:c>
+      <x:c r="D7" s="44" t="str">
+        <x:v>0.6679407284288028</x:v>
+      </x:c>
+      <x:c r="E7" s="44" t="str">
+        <x:v>0.5817003946763772</x:v>
+      </x:c>
+      <x:c r="F7" s="44" t="str">
+        <x:v>0.6103392335057061</x:v>
+      </x:c>
+      <x:c r="G7" s="44" t="str">
+        <x:v>0.8734436694178939</x:v>
+      </x:c>
+      <x:c r="H7" s="44" t="str">
+        <x:v>9.853879579997738</x:v>
+      </x:c>
+      <x:c r="I7" s="44" t="str">
+        <x:v>0.5054056380031398</x:v>
+      </x:c>
+      <x:c r="J7" s="44" t="str">
+        <x:v>0.0326700477054389</x:v>
+      </x:c>
+      <x:c r="K7" s="44" t="str">
+        <x:v>1.4949</x:v>
+      </x:c>
+      <x:c r="L7" s="50" t="str">
+        <x:v>390438</x:v>
+      </x:c>
+      <x:c r="M7" s="50" t="str">
         <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="42" t="str">
+        <x:v>CNN-BiLSTM</x:v>
+      </x:c>
+      <x:c r="B8" s="44" t="str">
+        <x:v>0.5270846800258565</x:v>
+      </x:c>
+      <x:c r="C8" s="44" t="str">
+        <x:v>0.5671460565237016</x:v>
+      </x:c>
+      <x:c r="D8" s="44" t="str">
+        <x:v>0.6649348577299911</x:v>
+      </x:c>
+      <x:c r="E8" s="44" t="str">
+        <x:v>0.5560753221633467</x:v>
+      </x:c>
+      <x:c r="F8" s="44" t="str">
+        <x:v>0.5428726689027361</x:v>
+      </x:c>
+      <x:c r="G8" s="44" t="str">
+        <x:v>0.8721893951509821</x:v>
+      </x:c>
+      <x:c r="H8" s="44" t="str">
+        <x:v>12.868202195997583</x:v>
+      </x:c>
+      <x:c r="I8" s="44" t="str">
+        <x:v>0.5209242119963164</x:v>
+      </x:c>
+      <x:c r="J8" s="44" t="str">
+        <x:v>0.03367318758864359</x:v>
+      </x:c>
+      <x:c r="K8" s="44" t="str">
+        <x:v>1.4834</x:v>
+      </x:c>
+      <x:c r="L8" s="50" t="str">
+        <x:v>387445</x:v>
+      </x:c>
+      <x:c r="M8" s="50" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
         <x:v>LSTM</x:v>
       </x:c>
-      <x:c r="B8" s="44" t="n">
+      <x:c r="B9" s="20" t="str">
         <x:v>0.5014221073044602</x:v>
       </x:c>
-      <x:c r="C8" s="44" t="n">
-        <x:v>0.2006594661340404</x:v>
-      </x:c>
-      <x:c r="D8" s="44" t="n">
+      <x:c r="C9" s="20" t="str">
+        <x:v>0.20064644266613882</x:v>
+      </x:c>
+      <x:c r="D9" s="20" t="str">
         <x:v>0.3298230660331335</x:v>
       </x:c>
-      <x:c r="E8" s="44" t="n">
-        <x:v>0.2203984092723267</x:v>
-      </x:c>
-      <x:c r="F8" s="44" t="n">
-        <x:v>0.4520484551817517</x:v>
-      </x:c>
-      <x:c r="G8" s="44" t="n">
-        <x:v>0.68901154711966</x:v>
-      </x:c>
-      <x:c r="H8" s="44" t="n">
-        <x:v>7.8894265740000264</x:v>
-      </x:c>
-      <x:c r="I8" s="44" t="n">
-        <x:v>0.2992368349996468</x:v>
-      </x:c>
-      <x:c r="J8" s="44" t="n">
-        <x:v>0.0193430404007528</x:v>
-      </x:c>
-      <x:c r="K8" s="44" t="n">
+      <x:c r="E9" s="20" t="str">
+        <x:v>0.2203818310686433</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
+        <x:v>0.4520379477940907</x:v>
+      </x:c>
+      <x:c r="G9" s="20" t="str">
+        <x:v>0.6889905045500638</x:v>
+      </x:c>
+      <x:c r="H9" s="20" t="str">
+        <x:v>3.8865443260001484</x:v>
+      </x:c>
+      <x:c r="I9" s="20" t="str">
+        <x:v>0.22446415000013076</x:v>
+      </x:c>
+      <x:c r="J9" s="20" t="str">
+        <x:v>0.014509641241120282</x:v>
+      </x:c>
+      <x:c r="K9" s="20" t="str">
         <x:v>1.396</x:v>
       </x:c>
-      <x:c r="L8" s="44" t="n">
+      <x:c r="L9" s="18" t="str">
         <x:v>365237</x:v>
       </x:c>
-      <x:c r="M8" s="44" t="n">
+      <x:c r="M9" s="18" t="str">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="B9" s="20"/>
-      <x:c r="C9" s="20"/>
-      <x:c r="D9" s="20"/>
-      <x:c r="E9" s="20"/>
-      <x:c r="F9" s="20"/>
-      <x:c r="G9" s="20"/>
-      <x:c r="H9" s="20"/>
-      <x:c r="I9" s="20"/>
-      <x:c r="J9" s="20"/>
-      <x:c r="K9" s="20"/>
-      <x:c r="L9" s="20"/>
-      <x:c r="M9" s="20"/>
     </x:row>
     <x:row r="10">
       <x:c r="B10" s="20"/>
@@ -2899,10 +3184,22 @@
       </x:extLst>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E4:E9">
+    <x:cfRule type="colorScale" priority="2">
+      <x:colorScale>
+        <x:cfvo type="min"/>
+        <x:cfvo type="percentile" val="50"/>
+        <x:cfvo type="max"/>
+        <x:color rgb="FFD9EAF7"/>
+        <x:color rgb="FF5DADE2"/>
+        <x:color rgb="FF1B4F72"/>
+      </x:colorScale>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e21665457834d66"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b8880e0b6c4419e"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73de69d36e3940e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4bf064c84d14087"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -3711,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bfb8619cc4144f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fe85bab3b004f81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4026,7 +4323,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd052a73ad08a41bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898fef1fc85d4851"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -4273,7 +4570,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44898fc713a04a66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1bdfd0c7d4f4851"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4362,7 +4659,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1043b63d5a9242fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228f08b337c14e68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4650,7 +4947,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13f8c339bfd54fa3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5e0b2abb70147f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>